<commit_message>
obsolete client id removed
</commit_message>
<xml_diff>
--- a/lib/measures/ReportRetrofitImpacts/resources/optimization_updated.xlsx
+++ b/lib/measures/ReportRetrofitImpacts/resources/optimization_updated.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-7425" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="weights" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="values" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="weights" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="values" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
wall insulation measure testing script
</commit_message>
<xml_diff>
--- a/lib/measures/ReportRetrofitImpacts/resources/optimization_updated.xlsx
+++ b/lib/measures/ReportRetrofitImpacts/resources/optimization_updated.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-7425" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="weights" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="values" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="weights" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="values" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -592,7 +592,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5471.82</v>
+        <v>2842.334445246917</v>
       </c>
       <c r="C2" t="n">
         <v>3</v>

</xml_diff>